<commit_message>
Show boxes each hour and SKUs per packer.
Expand a packer (or open By hour) for Intra Hour boxes by clock hour
plus Boxes Packed SKUs for that shift. Intra has no SKU column, so the
two stay side by side rather than inventing an hour×SKU join.

Co-authored-by: dSFulfilment <dSFulfilment@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/fixtures/packer-shift/Intra_Hour_Floor_Performance.xlsx
+++ b/fixtures/packer-shift/Intra_Hour_Floor_Performance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-13 14:00</t>
+          <t>2026-08-13 08:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -445,13 +445,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-13 15:00</t>
+          <t>2026-08-13 09:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -460,26 +460,176 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-08-13 10:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Alice Smith</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bob Jones</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13 09:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bob Jones</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-13 10:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bob Jones</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-13 08:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Carol Lee</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-13 09:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Carol Lee</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>2026-08-13 14:00</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Alice Smith</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-13 15:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Alice Smith</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Bob Jones</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C12" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="5">
-      <c r="C5" t="n">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-13 14:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dan West</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-13 15:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dan West</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" t="n">
         <v>55</v>
       </c>
     </row>

</xml_diff>